<commit_message>
update check_block merge method and add some test examples
</commit_message>
<xml_diff>
--- a/contracts/ChainSwap/output_debug/block_with_error.xlsx
+++ b/contracts/ChainSwap/output_debug/block_with_error.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K24"/>
+  <dimension ref="A1:K25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -456,12 +456,12 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>forward_path</t>
+          <t>revert_blockID</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>error_message_blockID</t>
+          <t>cfg_path</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
@@ -511,22 +511,22 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>['0x2e79B0xdaf', '0x2952B0xdaf', '0x30c8B0x2952B0xdaf', '0x295fB0xdaf']</t>
+          <t>0xde0</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>0x295fB0xdaf</t>
+          <t>['0xdaf', '0x2e79B0xdaf', '0x2952B0xdaf', '0x30c8B0x2952B0xdaf', '0x295fB0xdaf', '0x2e92B0xdaf', '0xde0']</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>['0x2987S0xdaf']</t>
+          <t>['0xdd4', '0x2e89S0xdaf', '0x30cdS0x2952S0xdaf', '0x2987S0xdaf']</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>[{'mstore_stmtID': '0x2987S0xdaf', 'value_var': '0x2962V0xdaf', 'value': '0x77697468647261776e20616c7265616479000000000000000000000000000000', 'decoded_chunk': 'withdrawn already', 'status': 'decoded'}]</t>
+          <t>[{'blockID': '0xdaf', 'mstore_stmtID': '0xdd4', 'value_var': '0xdb2', 'value': '0x8c379a000000000000000000000000000000000000000000000000000000000', 'decoded_chunk': None, 'status': 'not_string_constant'}, {'blockID': '0x2e79B0xdaf', 'mstore_stmtID': '0x2e89S0xdaf', 'value_var': '0x2e84V0xdaf', 'value': '0x20', 'decoded_chunk': None, 'status': 'not_string_constant'}, {'blockID': '0x30c8B0x2952B0xdaf', 'mstore_stmtID': '0x30cdS0x2952S0xdaf', 'value_var': '0x2958V0xdaf', 'value': '0x11', 'decoded_chunk': None, 'status': 'not_string_constant'}, {'blockID': '0x295fB0xdaf', 'mstore_stmtID': '0x2987S0xdaf', 'value_var': '0x2962V0xdaf', 'value': '0x77697468647261776e20616c7265616479000000000000000000000000000000', 'decoded_chunk': 'withdrawn already', 'status': 'decoded'}]</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -566,22 +566,22 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>['0x2dd9B0xec2', '0x27d2B0xec2', '0x30c8B0x27d2B0xec2', '0x27dfB0xec2']</t>
+          <t>0xef3</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>0x27dfB0xec2</t>
+          <t>['0xec2', '0x2dd9B0xec2', '0x27d2B0xec2', '0x30c8B0x27d2B0xec2', '0x27dfB0xec2', '0x2df2B0xec2', '0xef3']</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>['0x2807S0xec2']</t>
+          <t>['0xee7', '0x2de9S0xec2', '0x30cdS0x27d2S0xec2', '0x2807S0xec2']</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>[{'mstore_stmtID': '0x2807S0xec2', 'value_var': '0x27e2V0xec2', 'value': '0x746f6f20666577207369676e6174757265730000000000000000000000000000', 'decoded_chunk': 'too few signatures', 'status': 'decoded'}]</t>
+          <t>[{'blockID': '0xec2', 'mstore_stmtID': '0xee7', 'value_var': '0xec5', 'value': '0x8c379a000000000000000000000000000000000000000000000000000000000', 'decoded_chunk': None, 'status': 'not_string_constant'}, {'blockID': '0x2dd9B0xec2', 'mstore_stmtID': '0x2de9S0xec2', 'value_var': '0x2de4V0xec2', 'value': '0x20', 'decoded_chunk': None, 'status': 'not_string_constant'}, {'blockID': '0x30c8B0x27d2B0xec2', 'mstore_stmtID': '0x30cdS0x27d2S0xec2', 'value_var': '0x27d8V0xec2', 'value': '0x12', 'decoded_chunk': None, 'status': 'not_string_constant'}, {'blockID': '0x27dfB0xec2', 'mstore_stmtID': '0x2807S0xec2', 'value_var': '0x27e2V0xec2', 'value': '0x746f6f20666577207369676e6174757265730000000000000000000000000000', 'decoded_chunk': 'too few signatures', 'status': 'decoded'}]</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -621,22 +621,22 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>['0x2e39B0xf75', '0x28d2B0xf75', '0x30c8B0x28d2B0xf75', '0x28dfB0xf75']</t>
+          <t>0xfa6</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>0x28dfB0xf75</t>
+          <t>['0xf75', '0x2e39B0xf75', '0x28d2B0xf75', '0x30c8B0x28d2B0xf75', '0x28dfB0xf75', '0x2e52B0xf75', '0xfa6']</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>['0x2907S0xf75']</t>
+          <t>['0xf9a', '0x2e49S0xf75', '0x30cdS0x28d2S0xf75', '0x2907S0xf75']</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>[{'mstore_stmtID': '0x2907S0xf75', 'value_var': '0x28e2V0xf75', 'value': '0x72657065746974697665207369676e61746f7279000000000000000000000000', 'decoded_chunk': 'repetitive signatory', 'status': 'decoded'}]</t>
+          <t>[{'blockID': '0xf75', 'mstore_stmtID': '0xf9a', 'value_var': '0xf78', 'value': '0x8c379a000000000000000000000000000000000000000000000000000000000', 'decoded_chunk': None, 'status': 'not_string_constant'}, {'blockID': '0x2e39B0xf75', 'mstore_stmtID': '0x2e49S0xf75', 'value_var': '0x2e44V0xf75', 'value': '0x20', 'decoded_chunk': None, 'status': 'not_string_constant'}, {'blockID': '0x30c8B0x28d2B0xf75', 'mstore_stmtID': '0x30cdS0x28d2S0xf75', 'value_var': '0x28d8V0xf75', 'value': '0x14', 'decoded_chunk': None, 'status': 'not_string_constant'}, {'blockID': '0x28dfB0xf75', 'mstore_stmtID': '0x2907S0xf75', 'value_var': '0x28e2V0xf75', 'value': '0x72657065746974697665207369676e61746f7279000000000000000000000000', 'decoded_chunk': 'repetitive signatory', 'status': 'decoded'}]</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -676,22 +676,22 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>['0x2db9B0x1126', '0x2792B0x1126', '0x30c8B0x2792B0x1126', '0x279fB0x1126']</t>
+          <t>0x1157</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>0x279fB0x1126</t>
+          <t>['0x1126', '0x2db9B0x1126', '0x2792B0x1126', '0x30c8B0x2792B0x1126', '0x279fB0x1126', '0x2dd2B0x1126', '0x1157']</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>['0x27c7S0x1126']</t>
+          <t>['0x114b', '0x2dc9S0x1126', '0x30cdS0x2792S0x1126', '0x27c7S0x1126']</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>[{'mstore_stmtID': '0x27c7S0x1126', 'value_var': '0x27a2V0x1126', 'value': '0x696e76616c6964207369676e6174757265000000000000000000000000000000', 'decoded_chunk': 'invalid signature', 'status': 'decoded'}]</t>
+          <t>[{'blockID': '0x1126', 'mstore_stmtID': '0x114b', 'value_var': '0x1129', 'value': '0x8c379a000000000000000000000000000000000000000000000000000000000', 'decoded_chunk': None, 'status': 'not_string_constant'}, {'blockID': '0x2db9B0x1126', 'mstore_stmtID': '0x2dc9S0x1126', 'value_var': '0x2dc4V0x1126', 'value': '0x20', 'decoded_chunk': None, 'status': 'not_string_constant'}, {'blockID': '0x30c8B0x2792B0x1126', 'mstore_stmtID': '0x30cdS0x2792S0x1126', 'value_var': '0x2798V0x1126', 'value': '0x11', 'decoded_chunk': None, 'status': 'not_string_constant'}, {'blockID': '0x279fB0x1126', 'mstore_stmtID': '0x27c7S0x1126', 'value_var': '0x27a2V0x1126', 'value': '0x696e76616c6964207369676e6174757265000000000000000000000000000000', 'decoded_chunk': 'invalid signature', 'status': 'decoded'}]</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -731,22 +731,22 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>['0x2e99B0x11ab', '0x2992B0x11ab', '0x30c8B0x2992B0x11ab', '0x299fB0x11ab']</t>
+          <t>0x11dc</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>0x299fB0x11ab</t>
+          <t>['0x11ab', '0x2e99B0x11ab', '0x2992B0x11ab', '0x30c8B0x2992B0x11ab', '0x299fB0x11ab', '0x2eb2B0x11ab', '0x11dc']</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>['0x29c7S0x11ab']</t>
+          <t>['0x11d0', '0x2ea9S0x11ab', '0x30cdS0x2992S0x11ab', '0x29c7S0x11ab']</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>[{'mstore_stmtID': '0x29c7S0x11ab', 'value_var': '0x29a2V0x11ab', 'value': '0x756e617574686f72697a65640000000000000000000000000000000000000000', 'decoded_chunk': 'unauthorized', 'status': 'decoded'}]</t>
+          <t>[{'blockID': '0x11ab', 'mstore_stmtID': '0x11d0', 'value_var': '0x11ae', 'value': '0x8c379a000000000000000000000000000000000000000000000000000000000', 'decoded_chunk': None, 'status': 'not_string_constant'}, {'blockID': '0x2e99B0x11ab', 'mstore_stmtID': '0x2ea9S0x11ab', 'value_var': '0x2ea4V0x11ab', 'value': '0x20', 'decoded_chunk': None, 'status': 'not_string_constant'}, {'blockID': '0x30c8B0x2992B0x11ab', 'mstore_stmtID': '0x30cdS0x2992S0x11ab', 'value_var': '0x2998V0x11ab', 'value': '0xc', 'decoded_chunk': None, 'status': 'not_string_constant'}, {'blockID': '0x299fB0x11ab', 'mstore_stmtID': '0x29c7S0x11ab', 'value_var': '0x29a2V0x11ab', 'value': '0x756e617574686f72697a65640000000000000000000000000000000000000000', 'decoded_chunk': 'unauthorized', 'status': 'decoded'}]</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -786,22 +786,22 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>['0x2eb9B0x1382', '0x29d2B0x1382', '0x30c8B0x29d2B0x1382', '0x29dfB0x1382']</t>
+          <t>0x13b3</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>0x29dfB0x1382</t>
+          <t>['0x1382', '0x2eb9B0x1382', '0x29d2B0x1382', '0x30c8B0x29d2B0x1382', '0x29dfB0x1382', '0x2ed2B0x1382', '0x13b3']</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>['0x2a07S0x1382', '0x2a2dS0x1382']</t>
+          <t>['0x13a7', '0x2ec9S0x1382', '0x30cdS0x29d2S0x1382', '0x2a07S0x1382', '0x2a2dS0x1382']</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>[{'mstore_stmtID': '0x2a07S0x1382', 'value_var': '0x29e2V0x1382', 'value': '0x436f6e747261637420696e7374616e63652068617320616c7265616479206265', 'decoded_chunk': 'Contract instance has already be', 'status': 'decoded'}, {'mstore_stmtID': '0x2a2dS0x1382', 'value_var': '0x2a08V0x1382', 'value': '0x656e20696e697469616c697a6564000000000000000000000000000000000000', 'decoded_chunk': 'en initialized', 'status': 'decoded'}]</t>
+          <t>[{'blockID': '0x1382', 'mstore_stmtID': '0x13a7', 'value_var': '0x1385', 'value': '0x8c379a000000000000000000000000000000000000000000000000000000000', 'decoded_chunk': None, 'status': 'not_string_constant'}, {'blockID': '0x2eb9B0x1382', 'mstore_stmtID': '0x2ec9S0x1382', 'value_var': '0x2ec4V0x1382', 'value': '0x20', 'decoded_chunk': None, 'status': 'not_string_constant'}, {'blockID': '0x30c8B0x29d2B0x1382', 'mstore_stmtID': '0x30cdS0x29d2S0x1382', 'value_var': '0x29d8V0x1382', 'value': '0x2e', 'decoded_chunk': None, 'status': 'not_string_constant'}, {'blockID': '0x29dfB0x1382', 'mstore_stmtID': '0x2a07S0x1382', 'value_var': '0x29e2V0x1382', 'value': '0x436f6e747261637420696e7374616e63652068617320616c7265616479206265', 'decoded_chunk': 'Contract instance has already be', 'status': 'decoded'}, {'blockID': '0x29dfB0x1382', 'mstore_stmtID': '0x2a2dS0x1382', 'value_var': '0x2a08V0x1382', 'value': '0x656e20696e697469616c697a6564000000000000000000000000000000000000', 'decoded_chunk': 'en initialized', 'status': 'decoded'}]</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -841,22 +841,22 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>['0x2e19B0x17ff', '0x2892B0x17ff', '0x30c8B0x2892B0x17ff', '0x289fB0x17ff']</t>
+          <t>0x1830</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>0x289fB0x17ff</t>
+          <t>['0x17ff', '0x2e19B0x17ff', '0x2892B0x17ff', '0x30c8B0x2892B0x17ff', '0x289fB0x17ff', '0x2e32B0x17ff', '0x1830']</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>['0x28c7S0x17ff']</t>
+          <t>['0x1824', '0x2e29S0x17ff', '0x30cdS0x2892S0x17ff', '0x28c7S0x17ff']</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>[{'mstore_stmtID': '0x28c7S0x17ff', 'value_var': '0x28a2V0x17ff', 'value': '0x66656520697320746f6f206c6f77000000000000000000000000000000000000', 'decoded_chunk': 'fee is too low', 'status': 'decoded'}]</t>
+          <t>[{'blockID': '0x17ff', 'mstore_stmtID': '0x1824', 'value_var': '0x1802', 'value': '0x8c379a000000000000000000000000000000000000000000000000000000000', 'decoded_chunk': None, 'status': 'not_string_constant'}, {'blockID': '0x2e19B0x17ff', 'mstore_stmtID': '0x2e29S0x17ff', 'value_var': '0x2e24V0x17ff', 'value': '0x20', 'decoded_chunk': None, 'status': 'not_string_constant'}, {'blockID': '0x30c8B0x2892B0x17ff', 'mstore_stmtID': '0x30cdS0x2892S0x17ff', 'value_var': '0x2898V0x17ff', 'value': '0xe', 'decoded_chunk': None, 'status': 'not_string_constant'}, {'blockID': '0x289fB0x17ff', 'mstore_stmtID': '0x28c7S0x17ff', 'value_var': '0x28a2V0x17ff', 'value': '0x66656520697320746f6f206c6f77000000000000000000000000000000000000', 'decoded_chunk': 'fee is too low', 'status': 'decoded'}]</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -896,22 +896,22 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>['0x2eb9B0x1abd', '0x29d2B0x1abd', '0x30c8B0x29d2B0x1abd', '0x29dfB0x1abd']</t>
+          <t>0x1aee</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>0x29dfB0x1abd</t>
+          <t>['0x1abd', '0x2eb9B0x1abd', '0x29d2B0x1abd', '0x30c8B0x29d2B0x1abd', '0x29dfB0x1abd', '0x2ed2B0x1abd', '0x1aee']</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>['0x2a07S0x1abd', '0x2a2dS0x1abd']</t>
+          <t>['0x1ae2', '0x2ec9S0x1abd', '0x30cdS0x29d2S0x1abd', '0x2a07S0x1abd', '0x2a2dS0x1abd']</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>[{'mstore_stmtID': '0x2a07S0x1abd', 'value_var': '0x29e2V0x1abd', 'value': '0x436f6e747261637420696e7374616e63652068617320616c7265616479206265', 'decoded_chunk': 'Contract instance has already be', 'status': 'decoded'}, {'mstore_stmtID': '0x2a2dS0x1abd', 'value_var': '0x2a08V0x1abd', 'value': '0x656e20696e697469616c697a6564000000000000000000000000000000000000', 'decoded_chunk': 'en initialized', 'status': 'decoded'}]</t>
+          <t>[{'blockID': '0x1abd', 'mstore_stmtID': '0x1ae2', 'value_var': '0x1ac0', 'value': '0x8c379a000000000000000000000000000000000000000000000000000000000', 'decoded_chunk': None, 'status': 'not_string_constant'}, {'blockID': '0x2eb9B0x1abd', 'mstore_stmtID': '0x2ec9S0x1abd', 'value_var': '0x2ec4V0x1abd', 'value': '0x20', 'decoded_chunk': None, 'status': 'not_string_constant'}, {'blockID': '0x30c8B0x29d2B0x1abd', 'mstore_stmtID': '0x30cdS0x29d2S0x1abd', 'value_var': '0x29d8V0x1abd', 'value': '0x2e', 'decoded_chunk': None, 'status': 'not_string_constant'}, {'blockID': '0x29dfB0x1abd', 'mstore_stmtID': '0x2a07S0x1abd', 'value_var': '0x29e2V0x1abd', 'value': '0x436f6e747261637420696e7374616e63652068617320616c7265616479206265', 'decoded_chunk': 'Contract instance has already be', 'status': 'decoded'}, {'blockID': '0x29dfB0x1abd', 'mstore_stmtID': '0x2a2dS0x1abd', 'value_var': '0x2a08V0x1abd', 'value': '0x656e20696e697469616c697a6564000000000000000000000000000000000000', 'decoded_chunk': 'en initialized', 'status': 'decoded'}]</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -951,22 +951,22 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>['0x2df9B0x1c6c', '0x2852B0x1c6c', '0x30c8B0x2852B0x1c6c', '0x285fB0x1c6c']</t>
+          <t>0x1c9d</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>0x285fB0x1c6c</t>
+          <t>['0x1c6c', '0x2df9B0x1c6c', '0x2852B0x1c6c', '0x30c8B0x2852B0x1c6c', '0x285fB0x1c6c', '0x2e12B0x1c6c', '0x1c9d']</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>['0x2887S0x1c6c']</t>
+          <t>['0x1c91', '0x2e09S0x1c6c', '0x30cdS0x2852S0x1c6c', '0x2887S0x1c6c']</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>[{'mstore_stmtID': '0x2887S0x1c6c', 'value_var': '0x2862V0x1c6c', 'value': '0x536166654d6174683a206164646974696f6e206f766572666c6f770000000000', 'decoded_chunk': 'SafeMath: addition overflow', 'status': 'decoded'}]</t>
+          <t>[{'blockID': '0x1c6c', 'mstore_stmtID': '0x1c91', 'value_var': '0x1c6f', 'value': '0x8c379a000000000000000000000000000000000000000000000000000000000', 'decoded_chunk': None, 'status': 'not_string_constant'}, {'blockID': '0x2df9B0x1c6c', 'mstore_stmtID': '0x2e09S0x1c6c', 'value_var': '0x2e04V0x1c6c', 'value': '0x20', 'decoded_chunk': None, 'status': 'not_string_constant'}, {'blockID': '0x30c8B0x2852B0x1c6c', 'mstore_stmtID': '0x30cdS0x2852S0x1c6c', 'value_var': '0x2858V0x1c6c', 'value': '0x1b', 'decoded_chunk': None, 'status': 'not_string_constant'}, {'blockID': '0x285fB0x1c6c', 'mstore_stmtID': '0x2887S0x1c6c', 'value_var': '0x2862V0x1c6c', 'value': '0x536166654d6174683a206164646974696f6e206f766572666c6f770000000000', 'decoded_chunk': 'SafeMath: addition overflow', 'status': 'decoded'}]</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -1006,50 +1006,50 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>['0x2d97B0x1fe9', '0x2759B0x1fe9', '0x3094B0x1fe9', '0x2764B0x1fe9']</t>
+          <t>0x201b</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>0x2764B0x1fe9</t>
+          <t>['0x1fe9', '0x2d97B0x1fe9', '0x2759B0x1fe9', '0x3094B0x1fe9', '0x2764B0x1fe9', '0x30c8B0x2764B0x1fe9', '0x276eB0x1fe9', '0x3143B0x276eB0x1fe9', '0x3146B0x276eB0x1fe9', '0x3161B0x276eB0x1fe9', '0x3c517B0x276eB0x1fe9', '0x277eB0x1fe9', '0x3180B0x1fe9', '0x2787B0x1fe9', '0x2db1B0x1fe9', '0x201b']</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['0x200e', '0x2da7S0x1fe9', '0x30cdS0x2764S0x1fe9']</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>[{'blockID': '0x1fe9', 'mstore_stmtID': '0x200e', 'value_var': '0x1fec', 'value': '0x8c379a000000000000000000000000000000000000000000000000000000000', 'decoded_chunk': None, 'status': 'not_string_constant'}, {'blockID': '0x2d97B0x1fe9', 'mstore_stmtID': '0x2da7S0x1fe9', 'value_var': '0x2da2V0x1fe9', 'value': '0x20', 'decoded_chunk': None, 'status': 'not_string_constant'}, {'blockID': '0x30c8B0x2764B0x1fe9', 'mstore_stmtID': '0x30cdS0x2764S0x1fe9', 'value_var': '0x3098V0x1fe9', 'value': '0x1e', 'decoded_chunk': None, 'status': 'not_string_constant'}]</t>
         </is>
       </c>
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr">
         <is>
-          <t>mstore_not_found</t>
+          <t>string_not_decoded</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>0x39b0xade</t>
+          <t>0x1fec</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>0xade0x39b</t>
+          <t>0x1fec</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>0xadb0x39b</t>
+          <t>0x1fe9</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0xa830x39b</t>
+          <t>0x1fdc</t>
         </is>
       </c>
       <c r="E12" t="b">
@@ -1057,54 +1057,50 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>['0x2f19B0xadb0x39b', '0x2adeB0xadb0x39b', '0x30c8B0x2adeB0xadb0x39b', '0x2aebB0xadb0x39b']</t>
+          <t>0x201b</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>0x2aebB0xadb0x39b</t>
+          <t>['0x1fe9', '0x2d97B0x1fe9', '0x2759B0x1fe9', '0x3094B0x1fe9', '0x2764B0x1fe9', '0x30c8B0x2764B0x1fe9', '0x276eB0x1fe9', '0x3143B0x276eB0x1fe9', '0x3146B0x276eB0x1fe9', '0x3161B0x276eB0x1fe9', '0x316aB0x276eB0x1fe9', '0x3c5f3B0x276eB0x1fe9', '0x277eB0x1fe9', '0x3180B0x1fe9', '0x2787B0x1fe9', '0x2db1B0x1fe9', '0x201b']</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>['0x2b13S0xadb0x39b']</t>
+          <t>['0x200e', '0x2da7S0x1fe9', '0x30cdS0x2764S0x1fe9', '0x316fS0x276eS0x1fe9']</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>[{'mstore_stmtID': '0x2b13S0xadb0x39b', 'value_var': '0x2aeeV0xadb0x39b', 'value': '0x4f6e6c792063616c6c656420627920466163746f727900000000000000000000', 'decoded_chunk': 'Only called by Factory', 'status': 'decoded'}]</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>Only called by Factory</t>
-        </is>
-      </c>
+          <t>[{'blockID': '0x1fe9', 'mstore_stmtID': '0x200e', 'value_var': '0x1fec', 'value': '0x8c379a000000000000000000000000000000000000000000000000000000000', 'decoded_chunk': None, 'status': 'not_string_constant'}, {'blockID': '0x2d97B0x1fe9', 'mstore_stmtID': '0x2da7S0x1fe9', 'value_var': '0x2da2V0x1fe9', 'value': '0x20', 'decoded_chunk': None, 'status': 'not_string_constant'}, {'blockID': '0x30c8B0x2764B0x1fe9', 'mstore_stmtID': '0x30cdS0x2764S0x1fe9', 'value_var': '0x3098V0x1fe9', 'value': '0x1e', 'decoded_chunk': None, 'status': 'not_string_constant'}, {'blockID': '0x316aB0x276eB0x1fe9', 'mstore_stmtID': '0x316fS0x276eS0x1fe9', 'value_var': '0x316aV0x276eV0x1fe9', 'value': '0x0', 'decoded_chunk': None, 'status': 'not_string_constant'}]</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr">
         <is>
-          <t>decoded</t>
+          <t>string_not_decoded</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>0x897V0x2ef</t>
+          <t>0x39b0xade</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>0x897S0x2ef</t>
+          <t>0xade0x39b</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>0x894B0x2ef</t>
+          <t>0xadb0x39b</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>0x88fB0x2ef</t>
+          <t>0xa830x39b</t>
         </is>
       </c>
       <c r="E13" t="b">
@@ -1112,27 +1108,27 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>['0x2eb9B0x894B0x2ef', '0x29d2B0x894B0x2ef', '0x30c8B0x29d2B0x894B0x2ef', '0x29dfB0x894B0x2ef']</t>
+          <t>0xb0c0x39b</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>0x29dfB0x894B0x2ef</t>
+          <t>['0xadb0x39b', '0x2f19B0xadb0x39b', '0x2adeB0xadb0x39b', '0x30c8B0x2adeB0xadb0x39b', '0x2aebB0xadb0x39b', '0x2f32B0xadb0x39b', '0xb0c0x39b']</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>['0x2a07S0x894S0x2ef', '0x2a2dS0x894S0x2ef']</t>
+          <t>['0xb000x39b', '0x2f29S0xadb0x39b', '0x30cdS0x2adeS0xadb0x39b', '0x2b13S0xadb0x39b']</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>[{'mstore_stmtID': '0x2a07S0x894S0x2ef', 'value_var': '0x29e2V0x894V0x2ef', 'value': '0x436f6e747261637420696e7374616e63652068617320616c7265616479206265', 'decoded_chunk': 'Contract instance has already be', 'status': 'decoded'}, {'mstore_stmtID': '0x2a2dS0x894S0x2ef', 'value_var': '0x2a08V0x894V0x2ef', 'value': '0x656e20696e697469616c697a6564000000000000000000000000000000000000', 'decoded_chunk': 'en initialized', 'status': 'decoded'}]</t>
+          <t>[{'blockID': '0xadb0x39b', 'mstore_stmtID': '0xb000x39b', 'value_var': '0x39b0xade', 'value': '0x8c379a000000000000000000000000000000000000000000000000000000000', 'decoded_chunk': None, 'status': 'not_string_constant'}, {'blockID': '0x2f19B0xadb0x39b', 'mstore_stmtID': '0x2f29S0xadb0x39b', 'value_var': '0x2f24V0xadb0x39b', 'value': '0x20', 'decoded_chunk': None, 'status': 'not_string_constant'}, {'blockID': '0x30c8B0x2adeB0xadb0x39b', 'mstore_stmtID': '0x30cdS0x2adeS0xadb0x39b', 'value_var': '0x2ae4V0xadb0x39b', 'value': '0x16', 'decoded_chunk': None, 'status': 'not_string_constant'}, {'blockID': '0x2aebB0xadb0x39b', 'mstore_stmtID': '0x2b13S0xadb0x39b', 'value_var': '0x2aeeV0xadb0x39b', 'value': '0x4f6e6c792063616c6c656420627920466163746f727900000000000000000000', 'decoded_chunk': 'Only called by Factory', 'status': 'decoded'}]</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>Contract instance has already been initialized</t>
+          <t>Only called by Factory</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -1144,22 +1140,22 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>0x95f0x9baV0x343</t>
+          <t>0x897V0x2ef</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>0x9ba0x95fS0x343</t>
+          <t>0x897S0x2ef</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>0x9b70x95fB0x343</t>
+          <t>0x894B0x2ef</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>0x95fB0x343</t>
+          <t>0x88fB0x2ef</t>
         </is>
       </c>
       <c r="E14" t="b">
@@ -1167,27 +1163,27 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>['0x2f19B0x9b70x95fB0x343', '0x2adeB0x9b70x95fB0x343', '0x30c8B0x2adeB0x9b70x95fB0x343', '0x2aebB0x9b70x95fB0x343']</t>
+          <t>0x8c5B0x2ef</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>0x2aebB0x9b70x95fB0x343</t>
+          <t>['0x894B0x2ef', '0x2eb9B0x894B0x2ef', '0x29d2B0x894B0x2ef', '0x30c8B0x29d2B0x894B0x2ef', '0x29dfB0x894B0x2ef', '0x2ed2B0x894B0x2ef', '0x8c5B0x2ef']</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>['0x2b13S0x9b70x95fS0x343']</t>
+          <t>['0x8b9S0x2ef', '0x2ec9S0x894S0x2ef', '0x30cdS0x29d2S0x894S0x2ef', '0x2a07S0x894S0x2ef', '0x2a2dS0x894S0x2ef']</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>[{'mstore_stmtID': '0x2b13S0x9b70x95fS0x343', 'value_var': '0x2aeeV0x9b70x95fV0x343', 'value': '0x4f6e6c792063616c6c656420627920466163746f727900000000000000000000', 'decoded_chunk': 'Only called by Factory', 'status': 'decoded'}]</t>
+          <t>[{'blockID': '0x894B0x2ef', 'mstore_stmtID': '0x8b9S0x2ef', 'value_var': '0x897V0x2ef', 'value': '0x8c379a000000000000000000000000000000000000000000000000000000000', 'decoded_chunk': None, 'status': 'not_string_constant'}, {'blockID': '0x2eb9B0x894B0x2ef', 'mstore_stmtID': '0x2ec9S0x894S0x2ef', 'value_var': '0x2ec4V0x894V0x2ef', 'value': '0x20', 'decoded_chunk': None, 'status': 'not_string_constant'}, {'blockID': '0x30c8B0x29d2B0x894B0x2ef', 'mstore_stmtID': '0x30cdS0x29d2S0x894S0x2ef', 'value_var': '0x29d8V0x894V0x2ef', 'value': '0x2e', 'decoded_chunk': None, 'status': 'not_string_constant'}, {'blockID': '0x29dfB0x894B0x2ef', 'mstore_stmtID': '0x2a07S0x894S0x2ef', 'value_var': '0x29e2V0x894V0x2ef', 'value': '0x436f6e747261637420696e7374616e63652068617320616c7265616479206265', 'decoded_chunk': 'Contract instance has already be', 'status': 'decoded'}, {'blockID': '0x29dfB0x894B0x2ef', 'mstore_stmtID': '0x2a2dS0x894S0x2ef', 'value_var': '0x2a08V0x894V0x2ef', 'value': '0x656e20696e697469616c697a6564000000000000000000000000000000000000', 'decoded_chunk': 'en initialized', 'status': 'decoded'}]</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>Only called by Factory</t>
+          <t>Contract instance has already been initialized</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -1199,22 +1195,22 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>0x1e91V0x1d32V0x1a19</t>
+          <t>0x95f0x9baV0x343</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>0x1e91S0x1d32S0x1a19</t>
+          <t>0x9ba0x95fS0x343</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>0x1e8eB0x1d32B0x1a19</t>
+          <t>0x9b70x95fB0x343</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>0x1e89B0x1d32B0x1a19</t>
+          <t>0x95fB0x343</t>
         </is>
       </c>
       <c r="E15" t="b">
@@ -1222,27 +1218,27 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>['0x2f39B0x1e8eB0x1d32B0x1a19', '0x2b1eB0x1e8eB0x1d32B0x1a19', '0x30c8B0x2b1eB0x1e8eB0x1d32B0x1a19', '0x2b2bB0x1e8eB0x1d32B0x1a19']</t>
+          <t>0x9e80x95fB0x343</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>0x2b2bB0x1e8eB0x1d32B0x1a19</t>
+          <t>['0x9b70x95fB0x343', '0x2f19B0x9b70x95fB0x343', '0x2adeB0x9b70x95fB0x343', '0x30c8B0x2adeB0x9b70x95fB0x343', '0x2aebB0x9b70x95fB0x343', '0x2f32B0x9b70x95fB0x343', '0x9e80x95fB0x343']</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>['0x2b53S0x1e8eS0x1d32S0x1a19']</t>
+          <t>['0x9dc0x95fS0x343', '0x2f29S0x9b70x95fS0x343', '0x30cdS0x2adeS0x9b70x95fS0x343', '0x2b13S0x9b70x95fS0x343']</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>[{'mstore_stmtID': '0x2b53S0x1e8eS0x1d32S0x1a19', 'value_var': '0x2b2eV0x1e8eV0x1d32V0x1a19', 'value': '0x5361666545524332303a2063616c6c20746f206e6f6e2d636f6e747261637400', 'decoded_chunk': 'SafeERC20: call to non-contract', 'status': 'decoded'}]</t>
+          <t>[{'blockID': '0x9b70x95fB0x343', 'mstore_stmtID': '0x9dc0x95fS0x343', 'value_var': '0x95f0x9baV0x343', 'value': '0x8c379a000000000000000000000000000000000000000000000000000000000', 'decoded_chunk': None, 'status': 'not_string_constant'}, {'blockID': '0x2f19B0x9b70x95fB0x343', 'mstore_stmtID': '0x2f29S0x9b70x95fS0x343', 'value_var': '0x2f24V0x9b70x95fV0x343', 'value': '0x20', 'decoded_chunk': None, 'status': 'not_string_constant'}, {'blockID': '0x30c8B0x2adeB0x9b70x95fB0x343', 'mstore_stmtID': '0x30cdS0x2adeS0x9b70x95fS0x343', 'value_var': '0x2ae4V0x9b70x95fV0x343', 'value': '0x16', 'decoded_chunk': None, 'status': 'not_string_constant'}, {'blockID': '0x2aebB0x9b70x95fB0x343', 'mstore_stmtID': '0x2b13S0x9b70x95fS0x343', 'value_var': '0x2aeeV0x9b70x95fV0x343', 'value': '0x4f6e6c792063616c6c656420627920466163746f727900000000000000000000', 'decoded_chunk': 'Only called by Factory', 'status': 'decoded'}]</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>SafeERC20: call to non-contract</t>
+          <t>Only called by Factory</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -1254,22 +1250,22 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>0x1f41V0x1d32V0x1a19</t>
+          <t>0x1e91V0x1d32V0x1a19</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>0x1f41S0x1d32S0x1a19</t>
+          <t>0x1e91S0x1d32S0x1a19</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>0x1f3eB0x1d32B0x1a19</t>
+          <t>0x1e8eB0x1d32B0x1a19</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>0x1f33B0x1d32B0x1a19</t>
+          <t>0x1e89B0x1d32B0x1a19</t>
         </is>
       </c>
       <c r="E16" t="b">
@@ -1277,27 +1273,27 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>['0x2e59B0x1f3eB0x1d32B0x1a19', '0x2912B0x1f3eB0x1d32B0x1a19', '0x30c8B0x2912B0x1f3eB0x1d32B0x1a19', '0x291fB0x1f3eB0x1d32B0x1a19']</t>
+          <t>0x1ebfB0x1d32B0x1a19</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>0x291fB0x1f3eB0x1d32B0x1a19</t>
+          <t>['0x1e8eB0x1d32B0x1a19', '0x2f39B0x1e8eB0x1d32B0x1a19', '0x2b1eB0x1e8eB0x1d32B0x1a19', '0x30c8B0x2b1eB0x1e8eB0x1d32B0x1a19', '0x2b2bB0x1e8eB0x1d32B0x1a19', '0x2f52B0x1e8eB0x1d32B0x1a19', '0x1ebfB0x1d32B0x1a19']</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>['0x2947S0x1f3eS0x1d32S0x1a19']</t>
+          <t>['0x1eb3S0x1d32S0x1a19', '0x2f49S0x1e8eS0x1d32S0x1a19', '0x30cdS0x2b1eS0x1e8eS0x1d32S0x1a19', '0x2b53S0x1e8eS0x1d32S0x1a19']</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>[{'mstore_stmtID': '0x2947S0x1f3eS0x1d32S0x1a19', 'value_var': '0x2922V0x1f3eV0x1d32V0x1a19', 'value': '0x5361666545524332303a206c6f772d6c6576656c2063616c6c206661696c6564', 'decoded_chunk': 'SafeERC20: low-level call failed', 'status': 'decoded'}]</t>
+          <t>[{'blockID': '0x1e8eB0x1d32B0x1a19', 'mstore_stmtID': '0x1eb3S0x1d32S0x1a19', 'value_var': '0x1e91V0x1d32V0x1a19', 'value': '0x8c379a000000000000000000000000000000000000000000000000000000000', 'decoded_chunk': None, 'status': 'not_string_constant'}, {'blockID': '0x2f39B0x1e8eB0x1d32B0x1a19', 'mstore_stmtID': '0x2f49S0x1e8eS0x1d32S0x1a19', 'value_var': '0x2f44V0x1e8eV0x1d32V0x1a19', 'value': '0x20', 'decoded_chunk': None, 'status': 'not_string_constant'}, {'blockID': '0x30c8B0x2b1eB0x1e8eB0x1d32B0x1a19', 'mstore_stmtID': '0x30cdS0x2b1eS0x1e8eS0x1d32S0x1a19', 'value_var': '0x2b24V0x1e8eV0x1d32V0x1a19', 'value': '0x1f', 'decoded_chunk': None, 'status': 'not_string_constant'}, {'blockID': '0x2b2bB0x1e8eB0x1d32B0x1a19', 'mstore_stmtID': '0x2b53S0x1e8eS0x1d32S0x1a19', 'value_var': '0x2b2eV0x1e8eV0x1d32V0x1a19', 'value': '0x5361666545524332303a2063616c6c20746f206e6f6e2d636f6e747261637400', 'decoded_chunk': 'SafeERC20: call to non-contract', 'status': 'decoded'}]</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>SafeERC20: low-level call failed</t>
+          <t>SafeERC20: call to non-contract</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -1309,22 +1305,22 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>0x1f9eV0x1d32V0x1a19</t>
+          <t>0x1f41V0x1d32V0x1a19</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>0x1f9eS0x1d32S0x1a19</t>
+          <t>0x1f41S0x1d32S0x1a19</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>0x1f9bB0x1d32B0x1a19</t>
+          <t>0x1f3eB0x1d32B0x1a19</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>0x1f96B0x1d32B0x1a19</t>
+          <t>0x1f33B0x1d32B0x1a19</t>
         </is>
       </c>
       <c r="E17" t="b">
@@ -1332,27 +1328,27 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>['0x2ef9B0x1f9bB0x1d32B0x1a19', '0x2a78B0x1f9bB0x1d32B0x1a19', '0x30c8B0x2a78B0x1f9bB0x1d32B0x1a19', '0x2a85B0x1f9bB0x1d32B0x1a19']</t>
+          <t>0x1f6fB0x1d32B0x1a19</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>0x2a85B0x1f9bB0x1d32B0x1a19</t>
+          <t>['0x1f3eB0x1d32B0x1a19', '0x2e59B0x1f3eB0x1d32B0x1a19', '0x2912B0x1f3eB0x1d32B0x1a19', '0x30c8B0x2912B0x1f3eB0x1d32B0x1a19', '0x291fB0x1f3eB0x1d32B0x1a19', '0x2e72B0x1f3eB0x1d32B0x1a19', '0x1f6fB0x1d32B0x1a19']</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>['0x2aadS0x1f9bS0x1d32S0x1a19', '0x2ad3S0x1f9bS0x1d32S0x1a19']</t>
+          <t>['0x1f63S0x1d32S0x1a19', '0x2e69S0x1f3eS0x1d32S0x1a19', '0x30cdS0x2912S0x1f3eS0x1d32S0x1a19', '0x2947S0x1f3eS0x1d32S0x1a19']</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>[{'mstore_stmtID': '0x2aadS0x1f9bS0x1d32S0x1a19', 'value_var': '0x2a88V0x1f9bV0x1d32V0x1a19', 'value': '0x5361666545524332303a204552433230206f7065726174696f6e20646964206e', 'decoded_chunk': 'SafeERC20: ERC20 operation did n', 'status': 'decoded'}, {'mstore_stmtID': '0x2ad3S0x1f9bS0x1d32S0x1a19', 'value_var': '0x2aaeV0x1f9bV0x1d32V0x1a19', 'value': '0x6f74207375636365656400000000000000000000000000000000000000000000', 'decoded_chunk': 'ot succeed', 'status': 'decoded'}]</t>
+          <t>[{'blockID': '0x1f3eB0x1d32B0x1a19', 'mstore_stmtID': '0x1f63S0x1d32S0x1a19', 'value_var': '0x1f41V0x1d32V0x1a19', 'value': '0x8c379a000000000000000000000000000000000000000000000000000000000', 'decoded_chunk': None, 'status': 'not_string_constant'}, {'blockID': '0x2e59B0x1f3eB0x1d32B0x1a19', 'mstore_stmtID': '0x2e69S0x1f3eS0x1d32S0x1a19', 'value_var': '0x2e64V0x1f3eV0x1d32V0x1a19', 'value': '0x20', 'decoded_chunk': None, 'status': 'not_string_constant'}, {'blockID': '0x30c8B0x2912B0x1f3eB0x1d32B0x1a19', 'mstore_stmtID': '0x30cdS0x2912S0x1f3eS0x1d32S0x1a19', 'value_var': '0x2918V0x1f3eV0x1d32V0x1a19', 'value': '0x20', 'decoded_chunk': None, 'status': 'not_string_constant'}, {'blockID': '0x291fB0x1f3eB0x1d32B0x1a19', 'mstore_stmtID': '0x2947S0x1f3eS0x1d32S0x1a19', 'value_var': '0x2922V0x1f3eV0x1d32V0x1a19', 'value': '0x5361666545524332303a206c6f772d6c6576656c2063616c6c206661696c6564', 'decoded_chunk': 'SafeERC20: low-level call failed', 'status': 'decoded'}]</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>SafeERC20: ERC20 operation did not succeed</t>
+          <t>SafeERC20: low-level call failed</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -1364,22 +1360,22 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>0x1e91V0x1e03V0x1cb8</t>
+          <t>0x1f9eV0x1d32V0x1a19</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>0x1e91S0x1e03S0x1cb8</t>
+          <t>0x1f9eS0x1d32S0x1a19</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>0x1e8eB0x1e03B0x1cb8</t>
+          <t>0x1f9bB0x1d32B0x1a19</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>0x1e89B0x1e03B0x1cb8</t>
+          <t>0x1f96B0x1d32B0x1a19</t>
         </is>
       </c>
       <c r="E18" t="b">
@@ -1387,27 +1383,27 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>['0x2f39B0x1e8eB0x1e03B0x1cb8', '0x2b1eB0x1e8eB0x1e03B0x1cb8', '0x30c8B0x2b1eB0x1e8eB0x1e03B0x1cb8', '0x2b2bB0x1e8eB0x1e03B0x1cb8']</t>
+          <t>0x1fccB0x1d32B0x1a19</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>0x2b2bB0x1e8eB0x1e03B0x1cb8</t>
+          <t>['0x1f9bB0x1d32B0x1a19', '0x2ef9B0x1f9bB0x1d32B0x1a19', '0x2a78B0x1f9bB0x1d32B0x1a19', '0x30c8B0x2a78B0x1f9bB0x1d32B0x1a19', '0x2a85B0x1f9bB0x1d32B0x1a19', '0x2f12B0x1f9bB0x1d32B0x1a19', '0x1fccB0x1d32B0x1a19']</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>['0x2b53S0x1e8eS0x1e03S0x1cb8']</t>
+          <t>['0x1fc0S0x1d32S0x1a19', '0x2f09S0x1f9bS0x1d32S0x1a19', '0x30cdS0x2a78S0x1f9bS0x1d32S0x1a19', '0x2aadS0x1f9bS0x1d32S0x1a19', '0x2ad3S0x1f9bS0x1d32S0x1a19']</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>[{'mstore_stmtID': '0x2b53S0x1e8eS0x1e03S0x1cb8', 'value_var': '0x2b2eV0x1e8eV0x1e03V0x1cb8', 'value': '0x5361666545524332303a2063616c6c20746f206e6f6e2d636f6e747261637400', 'decoded_chunk': 'SafeERC20: call to non-contract', 'status': 'decoded'}]</t>
+          <t>[{'blockID': '0x1f9bB0x1d32B0x1a19', 'mstore_stmtID': '0x1fc0S0x1d32S0x1a19', 'value_var': '0x1f9eV0x1d32V0x1a19', 'value': '0x8c379a000000000000000000000000000000000000000000000000000000000', 'decoded_chunk': None, 'status': 'not_string_constant'}, {'blockID': '0x2ef9B0x1f9bB0x1d32B0x1a19', 'mstore_stmtID': '0x2f09S0x1f9bS0x1d32S0x1a19', 'value_var': '0x2f04V0x1f9bV0x1d32V0x1a19', 'value': '0x20', 'decoded_chunk': None, 'status': 'not_string_constant'}, {'blockID': '0x30c8B0x2a78B0x1f9bB0x1d32B0x1a19', 'mstore_stmtID': '0x30cdS0x2a78S0x1f9bS0x1d32S0x1a19', 'value_var': '0x2a7eV0x1f9bV0x1d32V0x1a19', 'value': '0x2a', 'decoded_chunk': None, 'status': 'not_string_constant'}, {'blockID': '0x2a85B0x1f9bB0x1d32B0x1a19', 'mstore_stmtID': '0x2aadS0x1f9bS0x1d32S0x1a19', 'value_var': '0x2a88V0x1f9bV0x1d32V0x1a19', 'value': '0x5361666545524332303a204552433230206f7065726174696f6e20646964206e', 'decoded_chunk': 'SafeERC20: ERC20 operation did n', 'status': 'decoded'}, {'blockID': '0x2a85B0x1f9bB0x1d32B0x1a19', 'mstore_stmtID': '0x2ad3S0x1f9bS0x1d32S0x1a19', 'value_var': '0x2aaeV0x1f9bV0x1d32V0x1a19', 'value': '0x6f74207375636365656400000000000000000000000000000000000000000000', 'decoded_chunk': 'ot succeed', 'status': 'decoded'}]</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>SafeERC20: call to non-contract</t>
+          <t>SafeERC20: ERC20 operation did not succeed</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -1419,22 +1415,22 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>0x1f41V0x1e03V0x1cb8</t>
+          <t>0x1e91V0x1e03V0x1cb8</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>0x1f41S0x1e03S0x1cb8</t>
+          <t>0x1e91S0x1e03S0x1cb8</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>0x1f3eB0x1e03B0x1cb8</t>
+          <t>0x1e8eB0x1e03B0x1cb8</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>0x1f33B0x1e03B0x1cb8</t>
+          <t>0x1e89B0x1e03B0x1cb8</t>
         </is>
       </c>
       <c r="E19" t="b">
@@ -1442,27 +1438,27 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>['0x2e59B0x1f3eB0x1e03B0x1cb8', '0x2912B0x1f3eB0x1e03B0x1cb8', '0x30c8B0x2912B0x1f3eB0x1e03B0x1cb8', '0x291fB0x1f3eB0x1e03B0x1cb8']</t>
+          <t>0x1ebfB0x1e03B0x1cb8</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>0x291fB0x1f3eB0x1e03B0x1cb8</t>
+          <t>['0x1e8eB0x1e03B0x1cb8', '0x2f39B0x1e8eB0x1e03B0x1cb8', '0x2b1eB0x1e8eB0x1e03B0x1cb8', '0x30c8B0x2b1eB0x1e8eB0x1e03B0x1cb8', '0x2b2bB0x1e8eB0x1e03B0x1cb8', '0x2f52B0x1e8eB0x1e03B0x1cb8', '0x1ebfB0x1e03B0x1cb8']</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>['0x2947S0x1f3eS0x1e03S0x1cb8']</t>
+          <t>['0x1eb3S0x1e03S0x1cb8', '0x2f49S0x1e8eS0x1e03S0x1cb8', '0x30cdS0x2b1eS0x1e8eS0x1e03S0x1cb8', '0x2b53S0x1e8eS0x1e03S0x1cb8']</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>[{'mstore_stmtID': '0x2947S0x1f3eS0x1e03S0x1cb8', 'value_var': '0x2922V0x1f3eV0x1e03V0x1cb8', 'value': '0x5361666545524332303a206c6f772d6c6576656c2063616c6c206661696c6564', 'decoded_chunk': 'SafeERC20: low-level call failed', 'status': 'decoded'}]</t>
+          <t>[{'blockID': '0x1e8eB0x1e03B0x1cb8', 'mstore_stmtID': '0x1eb3S0x1e03S0x1cb8', 'value_var': '0x1e91V0x1e03V0x1cb8', 'value': '0x8c379a000000000000000000000000000000000000000000000000000000000', 'decoded_chunk': None, 'status': 'not_string_constant'}, {'blockID': '0x2f39B0x1e8eB0x1e03B0x1cb8', 'mstore_stmtID': '0x2f49S0x1e8eS0x1e03S0x1cb8', 'value_var': '0x2f44V0x1e8eV0x1e03V0x1cb8', 'value': '0x20', 'decoded_chunk': None, 'status': 'not_string_constant'}, {'blockID': '0x30c8B0x2b1eB0x1e8eB0x1e03B0x1cb8', 'mstore_stmtID': '0x30cdS0x2b1eS0x1e8eS0x1e03S0x1cb8', 'value_var': '0x2b24V0x1e8eV0x1e03V0x1cb8', 'value': '0x1f', 'decoded_chunk': None, 'status': 'not_string_constant'}, {'blockID': '0x2b2bB0x1e8eB0x1e03B0x1cb8', 'mstore_stmtID': '0x2b53S0x1e8eS0x1e03S0x1cb8', 'value_var': '0x2b2eV0x1e8eV0x1e03V0x1cb8', 'value': '0x5361666545524332303a2063616c6c20746f206e6f6e2d636f6e747261637400', 'decoded_chunk': 'SafeERC20: call to non-contract', 'status': 'decoded'}]</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>SafeERC20: low-level call failed</t>
+          <t>SafeERC20: call to non-contract</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -1474,22 +1470,22 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>0x1f9eV0x1e03V0x1cb8</t>
+          <t>0x1f41V0x1e03V0x1cb8</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>0x1f9eS0x1e03S0x1cb8</t>
+          <t>0x1f41S0x1e03S0x1cb8</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>0x1f9bB0x1e03B0x1cb8</t>
+          <t>0x1f3eB0x1e03B0x1cb8</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>0x1f96B0x1e03B0x1cb8</t>
+          <t>0x1f33B0x1e03B0x1cb8</t>
         </is>
       </c>
       <c r="E20" t="b">
@@ -1497,27 +1493,27 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>['0x2ef9B0x1f9bB0x1e03B0x1cb8', '0x2a78B0x1f9bB0x1e03B0x1cb8', '0x30c8B0x2a78B0x1f9bB0x1e03B0x1cb8', '0x2a85B0x1f9bB0x1e03B0x1cb8']</t>
+          <t>0x1f6fB0x1e03B0x1cb8</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>0x2a85B0x1f9bB0x1e03B0x1cb8</t>
+          <t>['0x1f3eB0x1e03B0x1cb8', '0x2e59B0x1f3eB0x1e03B0x1cb8', '0x2912B0x1f3eB0x1e03B0x1cb8', '0x30c8B0x2912B0x1f3eB0x1e03B0x1cb8', '0x291fB0x1f3eB0x1e03B0x1cb8', '0x2e72B0x1f3eB0x1e03B0x1cb8', '0x1f6fB0x1e03B0x1cb8']</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>['0x2aadS0x1f9bS0x1e03S0x1cb8', '0x2ad3S0x1f9bS0x1e03S0x1cb8']</t>
+          <t>['0x1f63S0x1e03S0x1cb8', '0x2e69S0x1f3eS0x1e03S0x1cb8', '0x30cdS0x2912S0x1f3eS0x1e03S0x1cb8', '0x2947S0x1f3eS0x1e03S0x1cb8']</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>[{'mstore_stmtID': '0x2aadS0x1f9bS0x1e03S0x1cb8', 'value_var': '0x2a88V0x1f9bV0x1e03V0x1cb8', 'value': '0x5361666545524332303a204552433230206f7065726174696f6e20646964206e', 'decoded_chunk': 'SafeERC20: ERC20 operation did n', 'status': 'decoded'}, {'mstore_stmtID': '0x2ad3S0x1f9bS0x1e03S0x1cb8', 'value_var': '0x2aaeV0x1f9bV0x1e03V0x1cb8', 'value': '0x6f74207375636365656400000000000000000000000000000000000000000000', 'decoded_chunk': 'ot succeed', 'status': 'decoded'}]</t>
+          <t>[{'blockID': '0x1f3eB0x1e03B0x1cb8', 'mstore_stmtID': '0x1f63S0x1e03S0x1cb8', 'value_var': '0x1f41V0x1e03V0x1cb8', 'value': '0x8c379a000000000000000000000000000000000000000000000000000000000', 'decoded_chunk': None, 'status': 'not_string_constant'}, {'blockID': '0x2e59B0x1f3eB0x1e03B0x1cb8', 'mstore_stmtID': '0x2e69S0x1f3eS0x1e03S0x1cb8', 'value_var': '0x2e64V0x1f3eV0x1e03V0x1cb8', 'value': '0x20', 'decoded_chunk': None, 'status': 'not_string_constant'}, {'blockID': '0x30c8B0x2912B0x1f3eB0x1e03B0x1cb8', 'mstore_stmtID': '0x30cdS0x2912S0x1f3eS0x1e03S0x1cb8', 'value_var': '0x2918V0x1f3eV0x1e03V0x1cb8', 'value': '0x20', 'decoded_chunk': None, 'status': 'not_string_constant'}, {'blockID': '0x291fB0x1f3eB0x1e03B0x1cb8', 'mstore_stmtID': '0x2947S0x1f3eS0x1e03S0x1cb8', 'value_var': '0x2922V0x1f3eV0x1e03V0x1cb8', 'value': '0x5361666545524332303a206c6f772d6c6576656c2063616c6c206661696c6564', 'decoded_chunk': 'SafeERC20: low-level call failed', 'status': 'decoded'}]</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>SafeERC20: ERC20 operation did not succeed</t>
+          <t>SafeERC20: low-level call failed</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -1529,22 +1525,22 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>0x5c6V0x1ef</t>
+          <t>0x1f9eV0x1e03V0x1cb8</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>0x5c6S0x1ef</t>
+          <t>0x1f9eS0x1e03S0x1cb8</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>0x5c3B0x1ef</t>
+          <t>0x1f9bB0x1e03B0x1cb8</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>0x5b7B0x1ef</t>
+          <t>0x1f96B0x1e03B0x1cb8</t>
         </is>
       </c>
       <c r="E21" t="b">
@@ -1552,27 +1548,27 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>['0x2ed9B0x5c3B0x1ef', '0x2a38B0x5c3B0x1ef', '0x30c8B0x2a38B0x5c3B0x1ef', '0x2a45B0x5c3B0x1ef']</t>
+          <t>0x1fccB0x1e03B0x1cb8</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>0x2a45B0x5c3B0x1ef</t>
+          <t>['0x1f9bB0x1e03B0x1cb8', '0x2ef9B0x1f9bB0x1e03B0x1cb8', '0x2a78B0x1f9bB0x1e03B0x1cb8', '0x30c8B0x2a78B0x1f9bB0x1e03B0x1cb8', '0x2a85B0x1f9bB0x1e03B0x1cb8', '0x2f12B0x1f9bB0x1e03B0x1cb8', '0x1fccB0x1e03B0x1cb8']</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>['0x2a6dS0x5c3S0x1ef']</t>
+          <t>['0x1fc0S0x1e03S0x1cb8', '0x2f09S0x1f9bS0x1e03S0x1cb8', '0x30cdS0x2a78S0x1f9bS0x1e03S0x1cb8', '0x2aadS0x1f9bS0x1e03S0x1cb8', '0x2ad3S0x1f9bS0x1e03S0x1cb8']</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>[{'mstore_stmtID': '0x2a6dS0x5c3S0x1ef', 'value_var': '0x2a48V0x5c3V0x1ef', 'value': '0x74776f206172726179206c656e7468206e6f7420657175616c00000000000000', 'decoded_chunk': 'two array lenth not equal', 'status': 'decoded'}]</t>
+          <t>[{'blockID': '0x1f9bB0x1e03B0x1cb8', 'mstore_stmtID': '0x1fc0S0x1e03S0x1cb8', 'value_var': '0x1f9eV0x1e03V0x1cb8', 'value': '0x8c379a000000000000000000000000000000000000000000000000000000000', 'decoded_chunk': None, 'status': 'not_string_constant'}, {'blockID': '0x2ef9B0x1f9bB0x1e03B0x1cb8', 'mstore_stmtID': '0x2f09S0x1f9bS0x1e03S0x1cb8', 'value_var': '0x2f04V0x1f9bV0x1e03V0x1cb8', 'value': '0x20', 'decoded_chunk': None, 'status': 'not_string_constant'}, {'blockID': '0x30c8B0x2a78B0x1f9bB0x1e03B0x1cb8', 'mstore_stmtID': '0x30cdS0x2a78S0x1f9bS0x1e03S0x1cb8', 'value_var': '0x2a7eV0x1f9bV0x1e03V0x1cb8', 'value': '0x2a', 'decoded_chunk': None, 'status': 'not_string_constant'}, {'blockID': '0x2a85B0x1f9bB0x1e03B0x1cb8', 'mstore_stmtID': '0x2aadS0x1f9bS0x1e03S0x1cb8', 'value_var': '0x2a88V0x1f9bV0x1e03V0x1cb8', 'value': '0x5361666545524332303a204552433230206f7065726174696f6e20646964206e', 'decoded_chunk': 'SafeERC20: ERC20 operation did n', 'status': 'decoded'}, {'blockID': '0x2a85B0x1f9bB0x1e03B0x1cb8', 'mstore_stmtID': '0x2ad3S0x1f9bS0x1e03S0x1cb8', 'value_var': '0x2aaeV0x1f9bV0x1e03V0x1cb8', 'value': '0x6f74207375636365656400000000000000000000000000000000000000000000', 'decoded_chunk': 'ot succeed', 'status': 'decoded'}]</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>two array lenth not equal</t>
+          <t>SafeERC20: ERC20 operation did not succeed</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -1584,22 +1580,22 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>0xc54V0x455</t>
+          <t>0x5c6V0x1ef</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>0xc54S0x455</t>
+          <t>0x5c6S0x1ef</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>0xc51B0x455</t>
+          <t>0x5c3B0x1ef</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>0xc45B0x455</t>
+          <t>0x5b7B0x1ef</t>
         </is>
       </c>
       <c r="E22" t="b">
@@ -1607,22 +1603,22 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>['0x2ed9B0xc51B0x455', '0x2a38B0xc51B0x455', '0x30c8B0x2a38B0xc51B0x455', '0x2a45B0xc51B0x455']</t>
+          <t>0x5f4B0x1ef</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>0x2a45B0xc51B0x455</t>
+          <t>['0x5c3B0x1ef', '0x2ed9B0x5c3B0x1ef', '0x2a38B0x5c3B0x1ef', '0x30c8B0x2a38B0x5c3B0x1ef', '0x2a45B0x5c3B0x1ef', '0x2ef2B0x5c3B0x1ef', '0x5f4B0x1ef']</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>['0x2a6dS0xc51S0x455']</t>
+          <t>['0x5e8S0x1ef', '0x2ee9S0x5c3S0x1ef', '0x30cdS0x2a38S0x5c3S0x1ef', '0x2a6dS0x5c3S0x1ef']</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>[{'mstore_stmtID': '0x2a6dS0xc51S0x455', 'value_var': '0x2a48V0xc51V0x455', 'value': '0x74776f206172726179206c656e7468206e6f7420657175616c00000000000000', 'decoded_chunk': 'two array lenth not equal', 'status': 'decoded'}]</t>
+          <t>[{'blockID': '0x5c3B0x1ef', 'mstore_stmtID': '0x5e8S0x1ef', 'value_var': '0x5c6V0x1ef', 'value': '0x8c379a000000000000000000000000000000000000000000000000000000000', 'decoded_chunk': None, 'status': 'not_string_constant'}, {'blockID': '0x2ed9B0x5c3B0x1ef', 'mstore_stmtID': '0x2ee9S0x5c3S0x1ef', 'value_var': '0x2ee4V0x5c3V0x1ef', 'value': '0x20', 'decoded_chunk': None, 'status': 'not_string_constant'}, {'blockID': '0x30c8B0x2a38B0x5c3B0x1ef', 'mstore_stmtID': '0x30cdS0x2a38S0x5c3S0x1ef', 'value_var': '0x2a3eV0x5c3V0x1ef', 'value': '0x19', 'decoded_chunk': None, 'status': 'not_string_constant'}, {'blockID': '0x2a45B0x5c3B0x1ef', 'mstore_stmtID': '0x2a6dS0x5c3S0x1ef', 'value_var': '0x2a48V0x5c3V0x1ef', 'value': '0x74776f206172726179206c656e7468206e6f7420657175616c00000000000000', 'decoded_chunk': 'two array lenth not equal', 'status': 'decoded'}]</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
@@ -1639,22 +1635,22 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>0x5b70xadeV0x1ef</t>
+          <t>0xc54V0x455</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>0xade0x5b7S0x1ef</t>
+          <t>0xc54S0x455</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>0xadb0x5b7B0x1ef</t>
+          <t>0xc51B0x455</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>0xa830x5b7B0x1ef</t>
+          <t>0xc45B0x455</t>
         </is>
       </c>
       <c r="E23" t="b">
@@ -1662,27 +1658,27 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>['0x2f19B0xadb0x5b7B0x1ef', '0x2adeB0xadb0x5b7B0x1ef', '0x30c8B0x2adeB0xadb0x5b7B0x1ef', '0x2aebB0xadb0x5b7B0x1ef']</t>
+          <t>0xc82B0x455</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>0x2aebB0xadb0x5b7B0x1ef</t>
+          <t>['0xc51B0x455', '0x2ed9B0xc51B0x455', '0x2a38B0xc51B0x455', '0x30c8B0x2a38B0xc51B0x455', '0x2a45B0xc51B0x455', '0x2ef2B0xc51B0x455', '0xc82B0x455']</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>['0x2b13S0xadb0x5b7S0x1ef']</t>
+          <t>['0xc76S0x455', '0x2ee9S0xc51S0x455', '0x30cdS0x2a38S0xc51S0x455', '0x2a6dS0xc51S0x455']</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>[{'mstore_stmtID': '0x2b13S0xadb0x5b7S0x1ef', 'value_var': '0x2aeeV0xadb0x5b7V0x1ef', 'value': '0x4f6e6c792063616c6c656420627920466163746f727900000000000000000000', 'decoded_chunk': 'Only called by Factory', 'status': 'decoded'}]</t>
+          <t>[{'blockID': '0xc51B0x455', 'mstore_stmtID': '0xc76S0x455', 'value_var': '0xc54V0x455', 'value': '0x8c379a000000000000000000000000000000000000000000000000000000000', 'decoded_chunk': None, 'status': 'not_string_constant'}, {'blockID': '0x2ed9B0xc51B0x455', 'mstore_stmtID': '0x2ee9S0xc51S0x455', 'value_var': '0x2ee4V0xc51V0x455', 'value': '0x20', 'decoded_chunk': None, 'status': 'not_string_constant'}, {'blockID': '0x30c8B0x2a38B0xc51B0x455', 'mstore_stmtID': '0x30cdS0x2a38S0xc51S0x455', 'value_var': '0x2a3eV0xc51V0x455', 'value': '0x19', 'decoded_chunk': None, 'status': 'not_string_constant'}, {'blockID': '0x2a45B0xc51B0x455', 'mstore_stmtID': '0x2a6dS0xc51S0x455', 'value_var': '0x2a48V0xc51V0x455', 'value': '0x74776f206172726179206c656e7468206e6f7420657175616c00000000000000', 'decoded_chunk': 'two array lenth not equal', 'status': 'decoded'}]</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>Only called by Factory</t>
+          <t>two array lenth not equal</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -1694,53 +1690,108 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
+          <t>0x5b70xadeV0x1ef</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>0xade0x5b7S0x1ef</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>0xadb0x5b7B0x1ef</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>0xa830x5b7B0x1ef</t>
+        </is>
+      </c>
+      <c r="E24" t="b">
+        <v>1</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>0xb0c0x5b7B0x1ef</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>['0xadb0x5b7B0x1ef', '0x2f19B0xadb0x5b7B0x1ef', '0x2adeB0xadb0x5b7B0x1ef', '0x30c8B0x2adeB0xadb0x5b7B0x1ef', '0x2aebB0xadb0x5b7B0x1ef', '0x2f32B0xadb0x5b7B0x1ef', '0xb0c0x5b7B0x1ef']</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>['0xb000x5b7S0x1ef', '0x2f29S0xadb0x5b7S0x1ef', '0x30cdS0x2adeS0xadb0x5b7S0x1ef', '0x2b13S0xadb0x5b7S0x1ef']</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>[{'blockID': '0xadb0x5b7B0x1ef', 'mstore_stmtID': '0xb000x5b7S0x1ef', 'value_var': '0x5b70xadeV0x1ef', 'value': '0x8c379a000000000000000000000000000000000000000000000000000000000', 'decoded_chunk': None, 'status': 'not_string_constant'}, {'blockID': '0x2f19B0xadb0x5b7B0x1ef', 'mstore_stmtID': '0x2f29S0xadb0x5b7S0x1ef', 'value_var': '0x2f24V0xadb0x5b7V0x1ef', 'value': '0x20', 'decoded_chunk': None, 'status': 'not_string_constant'}, {'blockID': '0x30c8B0x2adeB0xadb0x5b7B0x1ef', 'mstore_stmtID': '0x30cdS0x2adeS0xadb0x5b7S0x1ef', 'value_var': '0x2ae4V0xadb0x5b7V0x1ef', 'value': '0x16', 'decoded_chunk': None, 'status': 'not_string_constant'}, {'blockID': '0x2aebB0xadb0x5b7B0x1ef', 'mstore_stmtID': '0x2b13S0xadb0x5b7S0x1ef', 'value_var': '0x2aeeV0xadb0x5b7V0x1ef', 'value': '0x4f6e6c792063616c6c656420627920466163746f727900000000000000000000', 'decoded_chunk': 'Only called by Factory', 'status': 'decoded'}]</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Only called by Factory</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>decoded</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
           <t>0xc450x9baV0x455</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B25" t="inlineStr">
         <is>
           <t>0x9ba0xc45S0x455</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C25" t="inlineStr">
         <is>
           <t>0x9b70xc45B0x455</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="D25" t="inlineStr">
         <is>
           <t>0x95f0xc45B0x455</t>
         </is>
       </c>
-      <c r="E24" t="b">
-        <v>1</v>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>['0x2f19B0x9b70xc45B0x455', '0x2adeB0x9b70xc45B0x455', '0x30c8B0x2adeB0x9b70xc45B0x455', '0x2aebB0x9b70xc45B0x455']</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>0x2aebB0x9b70xc45B0x455</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>['0x2b13S0x9b70xc45S0x455']</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>[{'mstore_stmtID': '0x2b13S0x9b70xc45S0x455', 'value_var': '0x2aeeV0x9b70xc45V0x455', 'value': '0x4f6e6c792063616c6c656420627920466163746f727900000000000000000000', 'decoded_chunk': 'Only called by Factory', 'status': 'decoded'}]</t>
-        </is>
-      </c>
-      <c r="J24" t="inlineStr">
+      <c r="E25" t="b">
+        <v>1</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>0x9e80xc45B0x455</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>['0x9b70xc45B0x455', '0x2f19B0x9b70xc45B0x455', '0x2adeB0x9b70xc45B0x455', '0x30c8B0x2adeB0x9b70xc45B0x455', '0x2aebB0x9b70xc45B0x455', '0x2f32B0x9b70xc45B0x455', '0x9e80xc45B0x455']</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>['0x9dc0xc45S0x455', '0x2f29S0x9b70xc45S0x455', '0x30cdS0x2adeS0x9b70xc45S0x455', '0x2b13S0x9b70xc45S0x455']</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>[{'blockID': '0x9b70xc45B0x455', 'mstore_stmtID': '0x9dc0xc45S0x455', 'value_var': '0xc450x9baV0x455', 'value': '0x8c379a000000000000000000000000000000000000000000000000000000000', 'decoded_chunk': None, 'status': 'not_string_constant'}, {'blockID': '0x2f19B0x9b70xc45B0x455', 'mstore_stmtID': '0x2f29S0x9b70xc45S0x455', 'value_var': '0x2f24V0x9b70xc45V0x455', 'value': '0x20', 'decoded_chunk': None, 'status': 'not_string_constant'}, {'blockID': '0x30c8B0x2adeB0x9b70xc45B0x455', 'mstore_stmtID': '0x30cdS0x2adeS0x9b70xc45S0x455', 'value_var': '0x2ae4V0x9b70xc45V0x455', 'value': '0x16', 'decoded_chunk': None, 'status': 'not_string_constant'}, {'blockID': '0x2aebB0x9b70xc45B0x455', 'mstore_stmtID': '0x2b13S0x9b70xc45S0x455', 'value_var': '0x2aeeV0x9b70xc45V0x455', 'value': '0x4f6e6c792063616c6c656420627920466163746f727900000000000000000000', 'decoded_chunk': 'Only called by Factory', 'status': 'decoded'}]</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
         <is>
           <t>Only called by Factory</t>
         </is>
       </c>
-      <c r="K24" t="inlineStr">
+      <c r="K25" t="inlineStr">
         <is>
           <t>decoded</t>
         </is>

</xml_diff>